<commit_message>
Actualizar entrega docente: WAN MikroTik A/B, presupuesto y PPT WAN-2
</commit_message>
<xml_diff>
--- a/Anexos/Presupuesto_Inventario.xlsx
+++ b/Anexos/Presupuesto_Inventario.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Rcc3c6f9bc1f64b50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partidas" sheetId="2" r:id="R59f1f5ff0e654e4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sedes" sheetId="3" r:id="R85825c4b3bd74876"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servidores" sheetId="4" r:id="Rddf58cffd15a4669"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Rb075a380b5b644fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partidas" sheetId="2" r:id="Rc9b82e0aaff64697"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sedes" sheetId="3" r:id="R5368d132f1974fa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servidores" sheetId="4" r:id="R1ba867e1df4b487a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -365,7 +365,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>23-10-2026. CLP con IVA. Proyecto ficticio, 23 sedes y 650 puestos.</x:v>
+        <x:v>24-10-2026. WAN-2. CLP con IVA. Proyecto ficticio, 23 sedes y 650 puestos.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -395,7 +395,7 @@
       </x:c>
       <x:c r="B6" s="11" t="n">
         <x:f>SUMIFS('Partidas'!$F$5:$F$52,'Partidas'!$A$5:$A$52,"A")</x:f>
-        <x:v>710667942</x:v>
+        <x:v>689173923</x:v>
       </x:c>
       <x:c r="C6" s="11" t="n">
         <x:f>SUMIFS('Partidas'!$F$5:$F$52,'Partidas'!$A$5:$A$52,"B")</x:f>
@@ -409,7 +409,7 @@
       </x:c>
       <x:c r="B7" s="11" t="n">
         <x:f>ROUND(B6*B18,0)</x:f>
-        <x:v>106600191</x:v>
+        <x:v>103376088</x:v>
       </x:c>
       <x:c r="C7" s="11" t="n">
         <x:f>ROUND(C6*C18,0)</x:f>
@@ -423,7 +423,7 @@
       </x:c>
       <x:c r="B8" s="17" t="n">
         <x:f>SUM(B6:B7)</x:f>
-        <x:v>817268133</x:v>
+        <x:v>792550011</x:v>
       </x:c>
       <x:c r="C8" s="17" t="n">
         <x:f>SUM(C6:C7)</x:f>
@@ -465,7 +465,7 @@
       </x:c>
       <x:c r="B11" s="17" t="n">
         <x:f>SUM(B8:B10)</x:f>
-        <x:v>1526153453</x:v>
+        <x:v>1501435331</x:v>
       </x:c>
       <x:c r="C11" s="17" t="n">
         <x:f>SUM(C8:C10)</x:f>
@@ -493,7 +493,7 @@
       </x:c>
       <x:c r="B13" s="11" t="n">
         <x:f>B8-B12</x:f>
-        <x:v>657268133</x:v>
+        <x:v>632550011</x:v>
       </x:c>
       <x:c r="C13" s="11" t="n">
         <x:f>C8-C12</x:f>
@@ -947,21 +947,21 @@
         <x:v>wan_ge</x:v>
       </x:c>
       <x:c r="C14" s="8" t="str">
-        <x:v>Distribuidor WAN gigabit</x:v>
+        <x:v>Distribuidor WAN MikroTik hEX E50UG, bridge VLAN</x:v>
       </x:c>
       <x:c r="D14" s="9" t="n">
         <x:v>45</x:v>
       </x:c>
       <x:c r="E14" s="10" t="n">
-        <x:v>531860</x:v>
+        <x:v>77048</x:v>
       </x:c>
       <x:c r="F14" s="11" t="n">
         <x:f>ROUND(D14*E14,0)</x:f>
-        <x:v>23933700</x:v>
+        <x:v>3467160</x:v>
       </x:c>
       <x:c r="G14" s="2"/>
       <x:c r="H14" s="8" t="str">
-        <x:v>https://www.spdigital.cl/cisco-catalyst-1300-8-port-ge-ext-ps/</x:v>
+        <x:v>https://mikrotik.com/product/hex_2024</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
@@ -972,21 +972,21 @@
         <x:v>wan_mgig</x:v>
       </x:c>
       <x:c r="C15" s="8" t="str">
-        <x:v>Distribuidor Starlink central multigigabit</x:v>
+        <x:v>Distribuidor WAN-A central MikroTik CRS310, bridge VLAN 2,5G</x:v>
       </x:c>
       <x:c r="D15" s="9" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E15" s="10" t="n">
-        <x:v>1308937.644</x:v>
+        <x:v>281459</x:v>
       </x:c>
       <x:c r="F15" s="11" t="n">
         <x:f>ROUND(D15*E15,0)</x:f>
-        <x:v>1308938</x:v>
+        <x:v>281459</x:v>
       </x:c>
       <x:c r="G15" s="2"/>
       <x:c r="H15" s="8" t="str">
-        <x:v>https://www.cdw.com/product/cisco-catalyst-1300-8mgp-2x-switch-8-ports-managed-rack-mountable/7877041</x:v>
+        <x:v>https://mikrotik.com/product/crs310_8g_2s_in</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">

</xml_diff>

<commit_message>
Completar cuatro accesos WAN en todas las sedes, incluida Casa Matriz
E6 conserva conectividad móvil y la presentación muestra respaldos sucesivos hasta WOM. WAN-3 concilia interfaces, túneles, inventario y presupuesto. Validación: 99 pruebas Node, 44 de navegador y 9.900 combinaciones del modelo.
</commit_message>
<xml_diff>
--- a/Anexos/Presupuesto_Inventario.xlsx
+++ b/Anexos/Presupuesto_Inventario.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Rb075a380b5b644fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partidas" sheetId="2" r:id="Rc9b82e0aaff64697"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sedes" sheetId="3" r:id="R5368d132f1974fa3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servidores" sheetId="4" r:id="R1ba867e1df4b487a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Rba4056e21c0a4d01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partidas" sheetId="2" r:id="Rf78a85ba9c424b5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sedes" sheetId="3" r:id="Rad991d878ff340dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servidores" sheetId="4" r:id="R25babeecf2d7419f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -365,7 +365,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>24-10-2026. WAN-2. CLP con IVA. Proyecto ficticio, 23 sedes y 650 puestos.</x:v>
+        <x:v>25-10-2026. WAN-3: cuatro WAN por sede. CLP con IVA. Proyecto ficticio, 23 sedes y 650 puestos.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -395,11 +395,11 @@
       </x:c>
       <x:c r="B6" s="11" t="n">
         <x:f>SUMIFS('Partidas'!$F$5:$F$52,'Partidas'!$A$5:$A$52,"A")</x:f>
-        <x:v>689173923</x:v>
+        <x:v>689675563</x:v>
       </x:c>
       <x:c r="C6" s="11" t="n">
         <x:f>SUMIFS('Partidas'!$F$5:$F$52,'Partidas'!$A$5:$A$52,"B")</x:f>
-        <x:v>244015297</x:v>
+        <x:v>244516937</x:v>
       </x:c>
       <x:c r="D6" s="2"/>
     </x:row>
@@ -409,11 +409,11 @@
       </x:c>
       <x:c r="B7" s="11" t="n">
         <x:f>ROUND(B6*B18,0)</x:f>
-        <x:v>103376088</x:v>
+        <x:v>103451334</x:v>
       </x:c>
       <x:c r="C7" s="11" t="n">
         <x:f>ROUND(C6*C18,0)</x:f>
-        <x:v>36602295</x:v>
+        <x:v>36677541</x:v>
       </x:c>
       <x:c r="D7" s="2"/>
     </x:row>
@@ -423,11 +423,11 @@
       </x:c>
       <x:c r="B8" s="17" t="n">
         <x:f>SUM(B6:B7)</x:f>
-        <x:v>792550011</x:v>
+        <x:v>793126897</x:v>
       </x:c>
       <x:c r="C8" s="17" t="n">
         <x:f>SUM(C6:C7)</x:f>
-        <x:v>280617592</x:v>
+        <x:v>281194478</x:v>
       </x:c>
       <x:c r="D8" s="2"/>
     </x:row>
@@ -437,11 +437,11 @@
       </x:c>
       <x:c r="B9" s="11" t="n">
         <x:f>B19*B20</x:f>
-        <x:v>658885320</x:v>
+        <x:v>660607380</x:v>
       </x:c>
       <x:c r="C9" s="11" t="n">
         <x:f>C19*C20</x:f>
-        <x:v>658885320</x:v>
+        <x:v>660607380</x:v>
       </x:c>
       <x:c r="D9" s="2"/>
     </x:row>
@@ -465,11 +465,11 @@
       </x:c>
       <x:c r="B11" s="17" t="n">
         <x:f>SUM(B8:B10)</x:f>
-        <x:v>1501435331</x:v>
+        <x:v>1503734277</x:v>
       </x:c>
       <x:c r="C11" s="17" t="n">
         <x:f>SUM(C8:C10)</x:f>
-        <x:v>964502912</x:v>
+        <x:v>966801858</x:v>
       </x:c>
       <x:c r="D11" s="2"/>
     </x:row>
@@ -493,11 +493,11 @@
       </x:c>
       <x:c r="B13" s="11" t="n">
         <x:f>B8-B12</x:f>
-        <x:v>632550011</x:v>
+        <x:v>633126897</x:v>
       </x:c>
       <x:c r="C13" s="11" t="n">
         <x:f>C8-C12</x:f>
-        <x:v>120617592</x:v>
+        <x:v>121194478</x:v>
       </x:c>
       <x:c r="D13" s="2"/>
     </x:row>
@@ -548,10 +548,10 @@
         <x:v>WAN mensual</x:v>
       </x:c>
       <x:c r="B19" s="10" t="n">
-        <x:v>10981422</x:v>
+        <x:v>11010123</x:v>
       </x:c>
       <x:c r="C19" s="10" t="n">
-        <x:v>10981422</x:v>
+        <x:v>11010123</x:v>
       </x:c>
       <x:c r="D19" s="2"/>
     </x:row>
@@ -1000,14 +1000,14 @@
         <x:v>CPE móvil Entel 5G, comprado</x:v>
       </x:c>
       <x:c r="D16" s="9" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E16" s="10" t="n">
         <x:v>342850</x:v>
       </x:c>
       <x:c r="F16" s="11" t="n">
         <x:f>ROUND(D16*E16,0)</x:f>
-        <x:v>7542700</x:v>
+        <x:v>7885550</x:v>
       </x:c>
       <x:c r="G16" s="2"/>
       <x:c r="H16" s="8" t="str">
@@ -1025,14 +1025,14 @@
         <x:v>CPE móvil WOM 4G, comprado</x:v>
       </x:c>
       <x:c r="D17" s="9" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E17" s="10" t="n">
         <x:v>158790</x:v>
       </x:c>
       <x:c r="F17" s="11" t="n">
         <x:f>ROUND(D17*E17,0)</x:f>
-        <x:v>3493380</x:v>
+        <x:v>3652170</x:v>
       </x:c>
       <x:c r="G17" s="2"/>
       <x:c r="H17" s="8" t="str">
@@ -1425,14 +1425,14 @@
         <x:v>CPE móvil Entel 5G, comprado</x:v>
       </x:c>
       <x:c r="D33" s="9" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E33" s="10" t="n">
         <x:v>342850</x:v>
       </x:c>
       <x:c r="F33" s="11" t="n">
         <x:f>ROUND(D33*E33,0)</x:f>
-        <x:v>7542700</x:v>
+        <x:v>7885550</x:v>
       </x:c>
       <x:c r="G33" s="2"/>
       <x:c r="H33" s="8" t="str">
@@ -1450,14 +1450,14 @@
         <x:v>CPE móvil WOM 4G, comprado</x:v>
       </x:c>
       <x:c r="D34" s="9" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E34" s="10" t="n">
         <x:v>158790</x:v>
       </x:c>
       <x:c r="F34" s="11" t="n">
         <x:f>ROUND(D34*E34,0)</x:f>
-        <x:v>3493380</x:v>
+        <x:v>3652170</x:v>
       </x:c>
       <x:c r="G34" s="2"/>
       <x:c r="H34" s="8" t="str">

</xml_diff>